<commit_message>
update stock analysis data
</commit_message>
<xml_diff>
--- a/output/stock_analysis_result.xlsx
+++ b/output/stock_analysis_result.xlsx
@@ -2756,16 +2756,16 @@
         </is>
       </c>
       <c r="M15" t="n">
-        <v>10382665</v>
+        <v>12157665</v>
       </c>
       <c r="N15" t="n">
-        <v>14081687</v>
+        <v>15856687</v>
       </c>
       <c r="O15" t="n">
-        <v>15353862</v>
+        <v>17128862</v>
       </c>
       <c r="P15" t="n">
-        <v>73677636</v>
+        <v>75452636</v>
       </c>
       <c r="Q15" t="n">
         <v>6968509</v>
@@ -2780,16 +2780,16 @@
         <v>20893849</v>
       </c>
       <c r="U15" t="n">
-        <v>2135000</v>
+        <v>3910000</v>
       </c>
       <c r="V15" t="n">
-        <v>16005479</v>
+        <v>17780479</v>
       </c>
       <c r="W15" t="n">
-        <v>30159510</v>
+        <v>31934510</v>
       </c>
       <c r="X15" t="n">
-        <v>48341024</v>
+        <v>50116024</v>
       </c>
       <c r="Y15" t="n">
         <v>1279156</v>
@@ -6570,16 +6570,16 @@
         </is>
       </c>
       <c r="M39" t="n">
-        <v>-1268957</v>
+        <v>-1121547</v>
       </c>
       <c r="N39" t="n">
-        <v>-1612961</v>
+        <v>-1465551</v>
       </c>
       <c r="O39" t="n">
-        <v>229471</v>
+        <v>376881</v>
       </c>
       <c r="P39" t="n">
-        <v>-26611906</v>
+        <v>-26464496</v>
       </c>
       <c r="Q39" t="n">
         <v>-1741460</v>
@@ -6594,16 +6594,16 @@
         <v>-11354606</v>
       </c>
       <c r="U39" t="n">
-        <v>183000</v>
+        <v>330410</v>
       </c>
       <c r="V39" t="n">
-        <v>869617</v>
+        <v>1017027</v>
       </c>
       <c r="W39" t="n">
-        <v>808617</v>
+        <v>956027</v>
       </c>
       <c r="X39" t="n">
-        <v>-13730943</v>
+        <v>-13583533</v>
       </c>
       <c r="Y39" t="n">
         <v>289503</v>
@@ -7047,16 +7047,16 @@
         </is>
       </c>
       <c r="M42" t="n">
-        <v>754872</v>
+        <v>729142</v>
       </c>
       <c r="N42" t="n">
-        <v>623232</v>
+        <v>597502</v>
       </c>
       <c r="O42" t="n">
-        <v>1748600</v>
+        <v>1722870</v>
       </c>
       <c r="P42" t="n">
-        <v>8316689</v>
+        <v>8290959</v>
       </c>
       <c r="Q42" t="n">
         <v>997028</v>
@@ -7071,16 +7071,16 @@
         <v>5840022</v>
       </c>
       <c r="U42" t="n">
-        <v>-457422</v>
+        <v>-483152</v>
       </c>
       <c r="V42" t="n">
-        <v>-370385</v>
+        <v>-396115</v>
       </c>
       <c r="W42" t="n">
-        <v>-206888</v>
+        <v>-232618</v>
       </c>
       <c r="X42" t="n">
-        <v>1872465</v>
+        <v>1846735</v>
       </c>
       <c r="Y42" t="n">
         <v>215266</v>
@@ -8319,16 +8319,16 @@
         </is>
       </c>
       <c r="M50" t="n">
-        <v>1685439</v>
+        <v>1650439</v>
       </c>
       <c r="N50" t="n">
-        <v>-194928</v>
+        <v>-229928</v>
       </c>
       <c r="O50" t="n">
-        <v>-1285174</v>
+        <v>-1320174</v>
       </c>
       <c r="P50" t="n">
-        <v>-8688966</v>
+        <v>-8723966</v>
       </c>
       <c r="Q50" t="n">
         <v>1779283</v>
@@ -8343,16 +8343,16 @@
         <v>-10956111</v>
       </c>
       <c r="U50" t="n">
-        <v>334000</v>
+        <v>299000</v>
       </c>
       <c r="V50" t="n">
-        <v>735000</v>
+        <v>700000</v>
       </c>
       <c r="W50" t="n">
-        <v>727406</v>
+        <v>692406</v>
       </c>
       <c r="X50" t="n">
-        <v>2621802</v>
+        <v>2586802</v>
       </c>
       <c r="Y50" t="n">
         <v>-427844</v>
@@ -13519,12 +13519,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2498.TW</t>
+          <t>8028.TW</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>宏達電</t>
+          <t>昇陽半導體</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -13533,28 +13533,28 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>40.2</v>
+        <v>233</v>
       </c>
       <c r="E83" t="n">
-        <v>39.89</v>
+        <v>227.2</v>
       </c>
       <c r="F83" t="n">
-        <v>40.44</v>
+        <v>233.35</v>
       </c>
       <c r="G83" t="n">
-        <v>40.54</v>
+        <v>239.65</v>
       </c>
       <c r="H83" t="n">
-        <v>3120072</v>
+        <v>3815963</v>
       </c>
       <c r="I83" t="n">
-        <v>2275002</v>
+        <v>2975215</v>
       </c>
       <c r="J83" t="n">
-        <v>43.3</v>
+        <v>256</v>
       </c>
       <c r="K83" t="n">
-        <v>39.2</v>
+        <v>216.5</v>
       </c>
       <c r="L83" t="inlineStr">
         <is>
@@ -13562,52 +13562,52 @@
         </is>
       </c>
       <c r="M83" t="n">
-        <v>577897</v>
+        <v>184684</v>
       </c>
       <c r="N83" t="n">
-        <v>-5854</v>
+        <v>-847501</v>
       </c>
       <c r="O83" t="n">
-        <v>-390500</v>
+        <v>-2423676</v>
       </c>
       <c r="P83" t="n">
-        <v>-5094141</v>
+        <v>-5700000</v>
       </c>
       <c r="Q83" t="n">
-        <v>330849</v>
+        <v>-1447130</v>
       </c>
       <c r="R83" t="n">
-        <v>-208514</v>
+        <v>-3294271</v>
       </c>
       <c r="S83" t="n">
-        <v>-525919</v>
+        <v>-4887144</v>
       </c>
       <c r="T83" t="n">
-        <v>-4817211</v>
+        <v>-8893544</v>
       </c>
       <c r="U83" t="n">
-        <v>0</v>
+        <v>1590000</v>
       </c>
       <c r="V83" t="n">
-        <v>0</v>
+        <v>2409000</v>
       </c>
       <c r="W83" t="n">
-        <v>0</v>
+        <v>2444000</v>
       </c>
       <c r="X83" t="n">
-        <v>-8000</v>
+        <v>3288000</v>
       </c>
       <c r="Y83" t="n">
-        <v>247048</v>
+        <v>41814</v>
       </c>
       <c r="Z83" t="n">
-        <v>202660</v>
+        <v>37770</v>
       </c>
       <c r="AA83" t="n">
-        <v>135419</v>
+        <v>19468</v>
       </c>
       <c r="AB83" t="n">
-        <v>-268930</v>
+        <v>-94456</v>
       </c>
       <c r="AC83" t="n">
         <v>-10</v>
@@ -13616,37 +13616,37 @@
         <v>-10</v>
       </c>
       <c r="AE83" t="n">
-        <v>-5</v>
+        <v>5</v>
       </c>
       <c r="AF83" t="n">
-        <v>-20</v>
+        <v>-30</v>
       </c>
       <c r="AG83" t="n">
         <v>0</v>
       </c>
       <c r="AH83" t="n">
-        <v>-30</v>
+        <v>-40</v>
       </c>
       <c r="AI83" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="AJ83" t="n">
-        <v>66.67</v>
+        <v>75</v>
       </c>
       <c r="AK83" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="AL83" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="AM83" t="inlineStr">
         <is>
-          <t>進場位置尚可</t>
+          <t>等待拉回確認</t>
         </is>
       </c>
       <c r="AN83" t="inlineStr">
         <is>
-          <t>DT尚未轉強、貼近5MA、位置偏低但需等轉強、量能溫和放大、分數明顯升溫</t>
+          <t>DT尚未轉強、貼近5MA、量能溫和放大、分數升溫過快</t>
         </is>
       </c>
       <c r="AO83" t="inlineStr">
@@ -13661,17 +13661,17 @@
       </c>
       <c r="AQ83" t="inlineStr">
         <is>
-          <t>站上5日線、空頭排列、量能溫和放大、接近20日低點</t>
+          <t>站上5日線、空頭排列、量能溫和放大</t>
         </is>
       </c>
       <c r="AR83" t="inlineStr">
         <is>
-          <t>5日法人賣超</t>
+          <t>5日法人明顯賣超、投信買外資賣</t>
         </is>
       </c>
       <c r="AS83" t="inlineStr">
         <is>
-          <t>風險偏高：站上5日線、空頭排列、量能溫和放大、接近20日低點、5日法人賣超。目前不適合積極追蹤，等待結構改善。</t>
+          <t>風險偏高：站上5日線、空頭排列、量能溫和放大、5日法人明顯賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
@@ -13996,12 +13996,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>6116.TW</t>
+          <t>2498.TW</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>彩晶</t>
+          <t>宏達電</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -14010,28 +14010,28 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>14.15</v>
+        <v>40.2</v>
       </c>
       <c r="E86" t="n">
-        <v>14.09</v>
+        <v>39.89</v>
       </c>
       <c r="F86" t="n">
-        <v>14.16</v>
+        <v>40.44</v>
       </c>
       <c r="G86" t="n">
-        <v>14.21</v>
+        <v>40.54</v>
       </c>
       <c r="H86" t="n">
-        <v>16856838</v>
+        <v>3120072</v>
       </c>
       <c r="I86" t="n">
-        <v>22268621</v>
+        <v>2275002</v>
       </c>
       <c r="J86" t="n">
-        <v>15.15</v>
+        <v>43.3</v>
       </c>
       <c r="K86" t="n">
-        <v>13.6</v>
+        <v>39.2</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -14039,28 +14039,28 @@
         </is>
       </c>
       <c r="M86" t="n">
-        <v>6093855</v>
+        <v>577897</v>
       </c>
       <c r="N86" t="n">
-        <v>4885111</v>
+        <v>-5854</v>
       </c>
       <c r="O86" t="n">
-        <v>-13388801</v>
+        <v>-390500</v>
       </c>
       <c r="P86" t="n">
-        <v>-11050586</v>
+        <v>-5094141</v>
       </c>
       <c r="Q86" t="n">
-        <v>5426269</v>
+        <v>330849</v>
       </c>
       <c r="R86" t="n">
-        <v>4589889</v>
+        <v>-208514</v>
       </c>
       <c r="S86" t="n">
-        <v>-13292258</v>
+        <v>-525919</v>
       </c>
       <c r="T86" t="n">
-        <v>-11251835</v>
+        <v>-4817211</v>
       </c>
       <c r="U86" t="n">
         <v>0</v>
@@ -14072,58 +14072,58 @@
         <v>0</v>
       </c>
       <c r="X86" t="n">
-        <v>0</v>
+        <v>-8000</v>
       </c>
       <c r="Y86" t="n">
-        <v>667586</v>
+        <v>247048</v>
       </c>
       <c r="Z86" t="n">
-        <v>295222</v>
+        <v>202660</v>
       </c>
       <c r="AA86" t="n">
-        <v>-96543</v>
+        <v>135419</v>
       </c>
       <c r="AB86" t="n">
-        <v>201249</v>
+        <v>-268930</v>
       </c>
       <c r="AC86" t="n">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="AD86" t="n">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="AE86" t="n">
-        <v>-15</v>
+        <v>-5</v>
       </c>
       <c r="AF86" t="n">
-        <v>-15</v>
+        <v>-20</v>
       </c>
       <c r="AG86" t="n">
         <v>0</v>
       </c>
       <c r="AH86" t="n">
-        <v>-34</v>
+        <v>-30</v>
       </c>
       <c r="AI86" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="AJ86" t="n">
-        <v>64.70999999999999</v>
+        <v>66.67</v>
       </c>
       <c r="AK86" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="AL86" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="AM86" t="inlineStr">
         <is>
-          <t>偏高或條件不足</t>
+          <t>進場位置尚可</t>
         </is>
       </c>
       <c r="AN86" t="inlineStr">
         <is>
-          <t>DT尚未轉強、貼近5MA、分數明顯升溫</t>
+          <t>DT尚未轉強、貼近5MA、位置偏低但需等轉強、量能溫和放大、分數明顯升溫</t>
         </is>
       </c>
       <c r="AO86" t="inlineStr">
@@ -14138,29 +14138,29 @@
       </c>
       <c r="AQ86" t="inlineStr">
         <is>
-          <t>站上5日線、空頭排列、量能未放大、接近20日低點</t>
+          <t>站上5日線、空頭排列、量能溫和放大、接近20日低點</t>
         </is>
       </c>
       <c r="AR86" t="inlineStr">
         <is>
-          <t>短線籌碼止穩、5日法人明顯賣超</t>
+          <t>5日法人賣超</t>
         </is>
       </c>
       <c r="AS86" t="inlineStr">
         <is>
-          <t>風險偏高：站上5日線、空頭排列、量能未放大、接近20日低點、短線籌碼止穩、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+          <t>風險偏高：站上5日線、空頭排列、量能溫和放大、接近20日低點、5日法人賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>6275.TWO</t>
+          <t>6116.TW</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>元山</t>
+          <t>彩晶</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -14169,28 +14169,28 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>44.85</v>
+        <v>14.15</v>
       </c>
       <c r="E87" t="n">
-        <v>45.12</v>
+        <v>14.09</v>
       </c>
       <c r="F87" t="n">
-        <v>45.61</v>
+        <v>14.16</v>
       </c>
       <c r="G87" t="n">
-        <v>45.41</v>
+        <v>14.21</v>
       </c>
       <c r="H87" t="n">
-        <v>78000</v>
+        <v>16856838</v>
       </c>
       <c r="I87" t="n">
-        <v>94000</v>
+        <v>22268621</v>
       </c>
       <c r="J87" t="n">
-        <v>48.9</v>
+        <v>15.15</v>
       </c>
       <c r="K87" t="n">
-        <v>43.65</v>
+        <v>13.6</v>
       </c>
       <c r="L87" t="inlineStr">
         <is>
@@ -14198,28 +14198,28 @@
         </is>
       </c>
       <c r="M87" t="n">
-        <v>0</v>
+        <v>6093855</v>
       </c>
       <c r="N87" t="n">
-        <v>0</v>
+        <v>4885111</v>
       </c>
       <c r="O87" t="n">
-        <v>0</v>
+        <v>-13388801</v>
       </c>
       <c r="P87" t="n">
-        <v>0</v>
+        <v>-11050586</v>
       </c>
       <c r="Q87" t="n">
-        <v>0</v>
+        <v>5426269</v>
       </c>
       <c r="R87" t="n">
-        <v>0</v>
+        <v>4589889</v>
       </c>
       <c r="S87" t="n">
-        <v>0</v>
+        <v>-13292258</v>
       </c>
       <c r="T87" t="n">
-        <v>0</v>
+        <v>-11251835</v>
       </c>
       <c r="U87" t="n">
         <v>0</v>
@@ -14234,16 +14234,16 @@
         <v>0</v>
       </c>
       <c r="Y87" t="n">
-        <v>0</v>
+        <v>667586</v>
       </c>
       <c r="Z87" t="n">
-        <v>0</v>
+        <v>295222</v>
       </c>
       <c r="AA87" t="n">
-        <v>0</v>
+        <v>-96543</v>
       </c>
       <c r="AB87" t="n">
-        <v>0</v>
+        <v>201249</v>
       </c>
       <c r="AC87" t="n">
         <v>-12</v>
@@ -14252,37 +14252,37 @@
         <v>-12</v>
       </c>
       <c r="AE87" t="n">
-        <v>-30</v>
+        <v>-15</v>
       </c>
       <c r="AF87" t="n">
-        <v>0</v>
+        <v>-15</v>
       </c>
       <c r="AG87" t="n">
         <v>0</v>
       </c>
       <c r="AH87" t="n">
-        <v>-12</v>
+        <v>-34</v>
       </c>
       <c r="AI87" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="AJ87" t="n">
-        <v>0</v>
+        <v>64.70999999999999</v>
       </c>
       <c r="AK87" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="AL87" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="AM87" t="inlineStr">
         <is>
-          <t>暫不追價</t>
+          <t>偏高或條件不足</t>
         </is>
       </c>
       <c r="AN87" t="inlineStr">
         <is>
-          <t>DT尚未轉強、尚未站上5MA、位置偏低但需等轉強</t>
+          <t>DT尚未轉強、貼近5MA、分數明顯升溫</t>
         </is>
       </c>
       <c r="AO87" t="inlineStr">
@@ -14297,29 +14297,29 @@
       </c>
       <c r="AQ87" t="inlineStr">
         <is>
-          <t>跌破5日線、量能未放大、接近20日低點</t>
+          <t>站上5日線、空頭排列、量能未放大、接近20日低點</t>
         </is>
       </c>
       <c r="AR87" t="inlineStr">
         <is>
-          <t>籌碼中性</t>
+          <t>短線籌碼止穩、5日法人明顯賣超</t>
         </is>
       </c>
       <c r="AS87" t="inlineStr">
         <is>
-          <t>風險偏高：跌破5日線、量能未放大、接近20日低點、籌碼中性。目前不適合積極追蹤，等待結構改善。</t>
+          <t>風險偏高：站上5日線、空頭排列、量能未放大、接近20日低點、短線籌碼止穩、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>3481.TW</t>
+          <t>6275.TWO</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>群創</t>
+          <t>元山</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -14328,28 +14328,28 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>48.7</v>
+        <v>44.85</v>
       </c>
       <c r="E88" t="n">
-        <v>48.04</v>
+        <v>45.12</v>
       </c>
       <c r="F88" t="n">
-        <v>48.57</v>
+        <v>45.61</v>
       </c>
       <c r="G88" t="n">
-        <v>47.97</v>
+        <v>45.41</v>
       </c>
       <c r="H88" t="n">
-        <v>99548905</v>
+        <v>78000</v>
       </c>
       <c r="I88" t="n">
-        <v>114045705</v>
+        <v>94000</v>
       </c>
       <c r="J88" t="n">
-        <v>52.4</v>
+        <v>48.9</v>
       </c>
       <c r="K88" t="n">
-        <v>44.95</v>
+        <v>43.65</v>
       </c>
       <c r="L88" t="inlineStr">
         <is>
@@ -14357,52 +14357,52 @@
         </is>
       </c>
       <c r="M88" t="n">
-        <v>26953397</v>
+        <v>0</v>
       </c>
       <c r="N88" t="n">
-        <v>19366389</v>
+        <v>0</v>
       </c>
       <c r="O88" t="n">
-        <v>-35408266</v>
+        <v>0</v>
       </c>
       <c r="P88" t="n">
-        <v>55520787</v>
+        <v>0</v>
       </c>
       <c r="Q88" t="n">
-        <v>20867981</v>
+        <v>0</v>
       </c>
       <c r="R88" t="n">
-        <v>14432255</v>
+        <v>0</v>
       </c>
       <c r="S88" t="n">
-        <v>-34510244</v>
+        <v>0</v>
       </c>
       <c r="T88" t="n">
-        <v>51643681</v>
+        <v>0</v>
       </c>
       <c r="U88" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="V88" t="n">
-        <v>4900</v>
+        <v>0</v>
       </c>
       <c r="W88" t="n">
-        <v>-111028</v>
+        <v>0</v>
       </c>
       <c r="X88" t="n">
-        <v>-396154</v>
+        <v>0</v>
       </c>
       <c r="Y88" t="n">
-        <v>6082416</v>
+        <v>0</v>
       </c>
       <c r="Z88" t="n">
-        <v>4929234</v>
+        <v>0</v>
       </c>
       <c r="AA88" t="n">
-        <v>-786994</v>
+        <v>0</v>
       </c>
       <c r="AB88" t="n">
-        <v>4273260</v>
+        <v>0</v>
       </c>
       <c r="AC88" t="n">
         <v>-12</v>
@@ -14411,35 +14411,37 @@
         <v>-12</v>
       </c>
       <c r="AE88" t="n">
-        <v>20</v>
+        <v>-30</v>
       </c>
       <c r="AF88" t="n">
-        <v>-50</v>
+        <v>0</v>
       </c>
       <c r="AG88" t="n">
         <v>0</v>
       </c>
       <c r="AH88" t="n">
-        <v>0</v>
+        <v>-12</v>
       </c>
       <c r="AI88" t="n">
-        <v>-12</v>
-      </c>
-      <c r="AJ88" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="AJ88" t="n">
+        <v>0</v>
+      </c>
       <c r="AK88" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="AL88" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="AM88" t="inlineStr">
         <is>
-          <t>偏高或條件不足</t>
+          <t>暫不追價</t>
         </is>
       </c>
       <c r="AN88" t="inlineStr">
         <is>
-          <t>DT尚未轉強、貼近5MA、位於20日區間中上緣、分數轉弱</t>
+          <t>DT尚未轉強、尚未站上5MA、位置偏低但需等轉強</t>
         </is>
       </c>
       <c r="AO88" t="inlineStr">
@@ -14454,29 +14456,29 @@
       </c>
       <c r="AQ88" t="inlineStr">
         <is>
-          <t>站上5日線、量能未放大</t>
+          <t>跌破5日線、量能未放大、接近20日低點</t>
         </is>
       </c>
       <c r="AR88" t="inlineStr">
         <is>
-          <t>5日法人明顯賣超、外資投信同步賣超</t>
+          <t>籌碼中性</t>
         </is>
       </c>
       <c r="AS88" t="inlineStr">
         <is>
-          <t>風險偏高：站上5日線、量能未放大、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
+          <t>風險偏高：跌破5日線、量能未放大、接近20日低點、籌碼中性。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2362.TW</t>
+          <t>3481.TW</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>藍天</t>
+          <t>群創</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -14485,28 +14487,28 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>47</v>
+        <v>48.7</v>
       </c>
       <c r="E89" t="n">
-        <v>46.93</v>
+        <v>48.04</v>
       </c>
       <c r="F89" t="n">
-        <v>47.5</v>
+        <v>48.57</v>
       </c>
       <c r="G89" t="n">
-        <v>47.84</v>
+        <v>47.97</v>
       </c>
       <c r="H89" t="n">
-        <v>358490</v>
+        <v>99548905</v>
       </c>
       <c r="I89" t="n">
-        <v>515193</v>
+        <v>114045705</v>
       </c>
       <c r="J89" t="n">
-        <v>49.9</v>
+        <v>52.4</v>
       </c>
       <c r="K89" t="n">
-        <v>46.25</v>
+        <v>44.95</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
@@ -14514,91 +14516,89 @@
         </is>
       </c>
       <c r="M89" t="n">
-        <v>30308</v>
+        <v>26953397</v>
       </c>
       <c r="N89" t="n">
-        <v>-116003</v>
+        <v>19366389</v>
       </c>
       <c r="O89" t="n">
-        <v>-410392</v>
+        <v>-35408266</v>
       </c>
       <c r="P89" t="n">
-        <v>-353753</v>
+        <v>55520787</v>
       </c>
       <c r="Q89" t="n">
-        <v>35211</v>
+        <v>20867981</v>
       </c>
       <c r="R89" t="n">
-        <v>-115907</v>
+        <v>14432255</v>
       </c>
       <c r="S89" t="n">
-        <v>-403100</v>
+        <v>-34510244</v>
       </c>
       <c r="T89" t="n">
-        <v>-352589</v>
+        <v>51643681</v>
       </c>
       <c r="U89" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="V89" t="n">
-        <v>0</v>
+        <v>4900</v>
       </c>
       <c r="W89" t="n">
-        <v>0</v>
+        <v>-111028</v>
       </c>
       <c r="X89" t="n">
-        <v>0</v>
+        <v>-396154</v>
       </c>
       <c r="Y89" t="n">
-        <v>-4903</v>
+        <v>6082416</v>
       </c>
       <c r="Z89" t="n">
-        <v>-96</v>
+        <v>4929234</v>
       </c>
       <c r="AA89" t="n">
-        <v>-7292</v>
+        <v>-786994</v>
       </c>
       <c r="AB89" t="n">
-        <v>-1164</v>
+        <v>4273260</v>
       </c>
       <c r="AC89" t="n">
-        <v>-14</v>
+        <v>-12</v>
       </c>
       <c r="AD89" t="n">
-        <v>-14</v>
+        <v>-12</v>
       </c>
       <c r="AE89" t="n">
-        <v>-15</v>
+        <v>20</v>
       </c>
       <c r="AF89" t="n">
-        <v>-20</v>
+        <v>-50</v>
       </c>
       <c r="AG89" t="n">
         <v>0</v>
       </c>
       <c r="AH89" t="n">
-        <v>-36</v>
+        <v>0</v>
       </c>
       <c r="AI89" t="n">
-        <v>22</v>
-      </c>
-      <c r="AJ89" t="n">
-        <v>61.11</v>
-      </c>
+        <v>-12</v>
+      </c>
+      <c r="AJ89" t="inlineStr"/>
       <c r="AK89" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="AL89" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="AM89" t="inlineStr">
         <is>
-          <t>等待拉回確認</t>
+          <t>偏高或條件不足</t>
         </is>
       </c>
       <c r="AN89" t="inlineStr">
         <is>
-          <t>DT尚未轉強、貼近5MA、位置偏低但需等轉強、分數明顯升溫</t>
+          <t>DT尚未轉強、貼近5MA、位於20日區間中上緣、分數轉弱</t>
         </is>
       </c>
       <c r="AO89" t="inlineStr">
@@ -14613,29 +14613,29 @@
       </c>
       <c r="AQ89" t="inlineStr">
         <is>
-          <t>站上5日線、空頭排列、量能未放大、接近20日低點</t>
+          <t>站上5日線、量能未放大</t>
         </is>
       </c>
       <c r="AR89" t="inlineStr">
         <is>
-          <t>5日法人賣超</t>
+          <t>5日法人明顯賣超、外資投信同步賣超</t>
         </is>
       </c>
       <c r="AS89" t="inlineStr">
         <is>
-          <t>風險偏高：站上5日線、空頭排列、量能未放大、接近20日低點、5日法人賣超。目前不適合積極追蹤，等待結構改善。</t>
+          <t>風險偏高：站上5日線、量能未放大、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>3163.TWO</t>
+          <t>2362.TW</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>波若威</t>
+          <t>藍天</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -14644,28 +14644,28 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>663</v>
+        <v>47</v>
       </c>
       <c r="E90" t="n">
-        <v>666.2</v>
+        <v>46.93</v>
       </c>
       <c r="F90" t="n">
-        <v>702.8</v>
+        <v>47.5</v>
       </c>
       <c r="G90" t="n">
-        <v>730.95</v>
+        <v>47.84</v>
       </c>
       <c r="H90" t="n">
-        <v>2048000</v>
+        <v>358490</v>
       </c>
       <c r="I90" t="n">
-        <v>1630200</v>
+        <v>515193</v>
       </c>
       <c r="J90" t="n">
-        <v>814</v>
+        <v>49.9</v>
       </c>
       <c r="K90" t="n">
-        <v>631</v>
+        <v>46.25</v>
       </c>
       <c r="L90" t="inlineStr">
         <is>
@@ -14673,28 +14673,28 @@
         </is>
       </c>
       <c r="M90" t="n">
-        <v>0</v>
+        <v>30308</v>
       </c>
       <c r="N90" t="n">
-        <v>0</v>
+        <v>-116003</v>
       </c>
       <c r="O90" t="n">
-        <v>0</v>
+        <v>-410392</v>
       </c>
       <c r="P90" t="n">
-        <v>0</v>
+        <v>-353753</v>
       </c>
       <c r="Q90" t="n">
-        <v>0</v>
+        <v>35211</v>
       </c>
       <c r="R90" t="n">
-        <v>0</v>
+        <v>-115907</v>
       </c>
       <c r="S90" t="n">
-        <v>0</v>
+        <v>-403100</v>
       </c>
       <c r="T90" t="n">
-        <v>0</v>
+        <v>-352589</v>
       </c>
       <c r="U90" t="n">
         <v>0</v>
@@ -14709,16 +14709,16 @@
         <v>0</v>
       </c>
       <c r="Y90" t="n">
-        <v>0</v>
+        <v>-4903</v>
       </c>
       <c r="Z90" t="n">
-        <v>0</v>
+        <v>-96</v>
       </c>
       <c r="AA90" t="n">
-        <v>0</v>
+        <v>-7292</v>
       </c>
       <c r="AB90" t="n">
-        <v>0</v>
+        <v>-1164</v>
       </c>
       <c r="AC90" t="n">
         <v>-14</v>
@@ -14727,37 +14727,37 @@
         <v>-14</v>
       </c>
       <c r="AE90" t="n">
-        <v>-35</v>
+        <v>-15</v>
       </c>
       <c r="AF90" t="n">
-        <v>0</v>
+        <v>-20</v>
       </c>
       <c r="AG90" t="n">
         <v>0</v>
       </c>
       <c r="AH90" t="n">
-        <v>-22</v>
+        <v>-36</v>
       </c>
       <c r="AI90" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="AJ90" t="n">
-        <v>36.36</v>
+        <v>61.11</v>
       </c>
       <c r="AK90" t="n">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="AL90" t="n">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="AM90" t="inlineStr">
         <is>
-          <t>暫不追價</t>
+          <t>等待拉回確認</t>
         </is>
       </c>
       <c r="AN90" t="inlineStr">
         <is>
-          <t>DT尚未轉強、尚未站上5MA、位置偏低但需等轉強、量能溫和放大、分數剛升溫</t>
+          <t>DT尚未轉強、貼近5MA、位置偏低但需等轉強、分數明顯升溫</t>
         </is>
       </c>
       <c r="AO90" t="inlineStr">
@@ -14772,29 +14772,29 @@
       </c>
       <c r="AQ90" t="inlineStr">
         <is>
-          <t>跌破5日線、空頭排列、量能溫和放大</t>
+          <t>站上5日線、空頭排列、量能未放大、接近20日低點</t>
         </is>
       </c>
       <c r="AR90" t="inlineStr">
         <is>
-          <t>籌碼中性</t>
+          <t>5日法人賣超</t>
         </is>
       </c>
       <c r="AS90" t="inlineStr">
         <is>
-          <t>風險偏高：跌破5日線、空頭排列、量能溫和放大、籌碼中性。目前不適合積極追蹤，等待結構改善。</t>
+          <t>風險偏高：站上5日線、空頭排列、量能未放大、接近20日低點、5日法人賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2308.TW</t>
+          <t>3163.TWO</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>台達電</t>
+          <t>波若威</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -14803,28 +14803,28 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>1710</v>
+        <v>663</v>
       </c>
       <c r="E91" t="n">
-        <v>1659</v>
+        <v>666.2</v>
       </c>
       <c r="F91" t="n">
-        <v>1733</v>
+        <v>702.8</v>
       </c>
       <c r="G91" t="n">
-        <v>1752.75</v>
+        <v>730.95</v>
       </c>
       <c r="H91" t="n">
-        <v>10673726</v>
+        <v>2048000</v>
       </c>
       <c r="I91" t="n">
-        <v>14272122</v>
+        <v>1630200</v>
       </c>
       <c r="J91" t="n">
-        <v>1885</v>
+        <v>814</v>
       </c>
       <c r="K91" t="n">
-        <v>1560</v>
+        <v>631</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -14832,91 +14832,91 @@
         </is>
       </c>
       <c r="M91" t="n">
-        <v>-571318</v>
+        <v>0</v>
       </c>
       <c r="N91" t="n">
-        <v>908777</v>
+        <v>0</v>
       </c>
       <c r="O91" t="n">
-        <v>-14199939</v>
+        <v>0</v>
       </c>
       <c r="P91" t="n">
-        <v>-10577853</v>
+        <v>0</v>
       </c>
       <c r="Q91" t="n">
-        <v>-844243</v>
+        <v>0</v>
       </c>
       <c r="R91" t="n">
-        <v>1310676</v>
+        <v>0</v>
       </c>
       <c r="S91" t="n">
-        <v>-10969822</v>
+        <v>0</v>
       </c>
       <c r="T91" t="n">
-        <v>-7109015</v>
+        <v>0</v>
       </c>
       <c r="U91" t="n">
-        <v>546888</v>
+        <v>0</v>
       </c>
       <c r="V91" t="n">
-        <v>-495960</v>
+        <v>0</v>
       </c>
       <c r="W91" t="n">
-        <v>-2694443</v>
+        <v>0</v>
       </c>
       <c r="X91" t="n">
-        <v>-3249403</v>
+        <v>0</v>
       </c>
       <c r="Y91" t="n">
-        <v>-273963</v>
+        <v>0</v>
       </c>
       <c r="Z91" t="n">
-        <v>94061</v>
+        <v>0</v>
       </c>
       <c r="AA91" t="n">
-        <v>-535674</v>
+        <v>0</v>
       </c>
       <c r="AB91" t="n">
-        <v>-219435</v>
+        <v>0</v>
       </c>
       <c r="AC91" t="n">
-        <v>-16</v>
+        <v>-14</v>
       </c>
       <c r="AD91" t="n">
-        <v>-16</v>
+        <v>-14</v>
       </c>
       <c r="AE91" t="n">
-        <v>-5</v>
+        <v>-35</v>
       </c>
       <c r="AF91" t="n">
-        <v>-35</v>
+        <v>0</v>
       </c>
       <c r="AG91" t="n">
         <v>0</v>
       </c>
       <c r="AH91" t="n">
-        <v>-34</v>
+        <v>-22</v>
       </c>
       <c r="AI91" t="n">
+        <v>8</v>
+      </c>
+      <c r="AJ91" t="n">
+        <v>36.36</v>
+      </c>
+      <c r="AK91" t="n">
         <v>18</v>
       </c>
-      <c r="AJ91" t="n">
-        <v>52.94</v>
-      </c>
-      <c r="AK91" t="n">
-        <v>45</v>
-      </c>
       <c r="AL91" t="n">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="AM91" t="inlineStr">
         <is>
-          <t>等待拉回確認</t>
+          <t>暫不追價</t>
         </is>
       </c>
       <c r="AN91" t="inlineStr">
         <is>
-          <t>DT尚未轉強、5MA乖離尚可、位於20日區間中上緣、分數明顯升溫</t>
+          <t>DT尚未轉強、尚未站上5MA、位置偏低但需等轉強、量能溫和放大、分數剛升溫</t>
         </is>
       </c>
       <c r="AO91" t="inlineStr">
@@ -14931,17 +14931,17 @@
       </c>
       <c r="AQ91" t="inlineStr">
         <is>
-          <t>站上5日線、空頭排列、量能未放大</t>
+          <t>跌破5日線、空頭排列、量能溫和放大</t>
         </is>
       </c>
       <c r="AR91" t="inlineStr">
         <is>
-          <t>短線籌碼止穩、5日法人明顯賣超、外資投信同步賣超</t>
+          <t>籌碼中性</t>
         </is>
       </c>
       <c r="AS91" t="inlineStr">
         <is>
-          <t>風險偏高：站上5日線、空頭排列、量能未放大、短線籌碼止穩、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
+          <t>風險偏高：跌破5日線、空頭排列、量能溫和放大、籌碼中性。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
@@ -15266,12 +15266,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>1718.TW</t>
+          <t>2308.TW</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>中纖</t>
+          <t>台達電</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -15280,28 +15280,28 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>10.5</v>
+        <v>1710</v>
       </c>
       <c r="E94" t="n">
-        <v>10.49</v>
+        <v>1659</v>
       </c>
       <c r="F94" t="n">
-        <v>10.54</v>
+        <v>1733</v>
       </c>
       <c r="G94" t="n">
-        <v>10.64</v>
+        <v>1752.75</v>
       </c>
       <c r="H94" t="n">
-        <v>6566522</v>
+        <v>10673726</v>
       </c>
       <c r="I94" t="n">
-        <v>9562776</v>
+        <v>14272122</v>
       </c>
       <c r="J94" t="n">
-        <v>11.95</v>
+        <v>1885</v>
       </c>
       <c r="K94" t="n">
-        <v>10.2</v>
+        <v>1560</v>
       </c>
       <c r="L94" t="inlineStr">
         <is>
@@ -15309,91 +15309,91 @@
         </is>
       </c>
       <c r="M94" t="n">
-        <v>1412080</v>
+        <v>-566318</v>
       </c>
       <c r="N94" t="n">
-        <v>3763377</v>
+        <v>913777</v>
       </c>
       <c r="O94" t="n">
-        <v>-622530</v>
+        <v>-14194939</v>
       </c>
       <c r="P94" t="n">
-        <v>4655722</v>
+        <v>-10572853</v>
       </c>
       <c r="Q94" t="n">
-        <v>1213977</v>
+        <v>-844243</v>
       </c>
       <c r="R94" t="n">
-        <v>3697418</v>
+        <v>1310676</v>
       </c>
       <c r="S94" t="n">
-        <v>-601588</v>
+        <v>-10969822</v>
       </c>
       <c r="T94" t="n">
-        <v>4937717</v>
+        <v>-7109015</v>
       </c>
       <c r="U94" t="n">
-        <v>0</v>
+        <v>551888</v>
       </c>
       <c r="V94" t="n">
-        <v>0</v>
+        <v>-490960</v>
       </c>
       <c r="W94" t="n">
-        <v>0</v>
+        <v>-2689443</v>
       </c>
       <c r="X94" t="n">
-        <v>-65000</v>
+        <v>-3244403</v>
       </c>
       <c r="Y94" t="n">
-        <v>198103</v>
+        <v>-273963</v>
       </c>
       <c r="Z94" t="n">
-        <v>65959</v>
+        <v>94061</v>
       </c>
       <c r="AA94" t="n">
-        <v>-20942</v>
+        <v>-535674</v>
       </c>
       <c r="AB94" t="n">
-        <v>-216995</v>
+        <v>-219435</v>
       </c>
       <c r="AC94" t="n">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="AD94" t="n">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="AE94" t="n">
-        <v>-15</v>
+        <v>-5</v>
       </c>
       <c r="AF94" t="n">
-        <v>-30</v>
+        <v>-35</v>
       </c>
       <c r="AG94" t="n">
         <v>0</v>
       </c>
       <c r="AH94" t="n">
-        <v>-10</v>
+        <v>-34</v>
       </c>
       <c r="AI94" t="n">
-        <v>-8</v>
+        <v>18</v>
       </c>
       <c r="AJ94" t="n">
-        <v>-80</v>
+        <v>52.94</v>
       </c>
       <c r="AK94" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="AL94" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="AM94" t="inlineStr">
         <is>
-          <t>暫不追價</t>
+          <t>等待拉回確認</t>
         </is>
       </c>
       <c r="AN94" t="inlineStr">
         <is>
-          <t>DT尚未轉強、貼近5MA、位置偏低但需等轉強、分數轉弱</t>
+          <t>DT尚未轉強、5MA乖離尚可、位於20日區間中上緣、分數明顯升溫</t>
         </is>
       </c>
       <c r="AO94" t="inlineStr">
@@ -15408,17 +15408,17 @@
       </c>
       <c r="AQ94" t="inlineStr">
         <is>
-          <t>站上5日線、空頭排列、量能未放大、接近20日低點</t>
+          <t>站上5日線、空頭排列、量能未放大</t>
         </is>
       </c>
       <c r="AR94" t="inlineStr">
         <is>
-          <t>5日法人明顯賣超</t>
+          <t>短線籌碼止穩、5日法人明顯賣超、外資投信同步賣超</t>
         </is>
       </c>
       <c r="AS94" t="inlineStr">
         <is>
-          <t>風險偏高：站上5日線、空頭排列、量能未放大、接近20日低點、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+          <t>風險偏高：站上5日線、空頭排列、量能未放大、短線籌碼止穩、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
@@ -15584,12 +15584,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>1303.TW</t>
+          <t>1718.TW</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>南亞</t>
+          <t>中纖</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -15598,28 +15598,28 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>224</v>
+        <v>10.5</v>
       </c>
       <c r="E96" t="n">
-        <v>231.6</v>
+        <v>10.49</v>
       </c>
       <c r="F96" t="n">
-        <v>230.65</v>
+        <v>10.54</v>
       </c>
       <c r="G96" t="n">
-        <v>221.12</v>
+        <v>10.64</v>
       </c>
       <c r="H96" t="n">
-        <v>48008257</v>
+        <v>6566522</v>
       </c>
       <c r="I96" t="n">
-        <v>53361085</v>
+        <v>9562776</v>
       </c>
       <c r="J96" t="n">
-        <v>250</v>
+        <v>11.95</v>
       </c>
       <c r="K96" t="n">
-        <v>174</v>
+        <v>10.2</v>
       </c>
       <c r="L96" t="inlineStr">
         <is>
@@ -15627,76 +15627,76 @@
         </is>
       </c>
       <c r="M96" t="n">
-        <v>-3809309</v>
+        <v>1412080</v>
       </c>
       <c r="N96" t="n">
-        <v>-22645671</v>
+        <v>3763377</v>
       </c>
       <c r="O96" t="n">
-        <v>-26959115</v>
+        <v>-622530</v>
       </c>
       <c r="P96" t="n">
-        <v>-37504582</v>
+        <v>4655722</v>
       </c>
       <c r="Q96" t="n">
-        <v>-6798444</v>
+        <v>1213977</v>
       </c>
       <c r="R96" t="n">
-        <v>-27265035</v>
+        <v>3697418</v>
       </c>
       <c r="S96" t="n">
-        <v>-33056760</v>
+        <v>-601588</v>
       </c>
       <c r="T96" t="n">
-        <v>-51665789</v>
+        <v>4937717</v>
       </c>
       <c r="U96" t="n">
-        <v>2714701</v>
+        <v>0</v>
       </c>
       <c r="V96" t="n">
-        <v>5618279</v>
+        <v>0</v>
       </c>
       <c r="W96" t="n">
-        <v>7877859</v>
+        <v>0</v>
       </c>
       <c r="X96" t="n">
-        <v>17968822</v>
+        <v>-65000</v>
       </c>
       <c r="Y96" t="n">
-        <v>274434</v>
+        <v>198103</v>
       </c>
       <c r="Z96" t="n">
-        <v>-998915</v>
+        <v>65959</v>
       </c>
       <c r="AA96" t="n">
-        <v>-1780214</v>
+        <v>-20942</v>
       </c>
       <c r="AB96" t="n">
-        <v>-3807615</v>
+        <v>-216995</v>
       </c>
       <c r="AC96" t="n">
-        <v>-20</v>
+        <v>-18</v>
       </c>
       <c r="AD96" t="n">
-        <v>-20</v>
+        <v>-18</v>
       </c>
       <c r="AE96" t="n">
-        <v>5</v>
+        <v>-15</v>
       </c>
       <c r="AF96" t="n">
-        <v>-55</v>
+        <v>-30</v>
       </c>
       <c r="AG96" t="n">
         <v>0</v>
       </c>
       <c r="AH96" t="n">
-        <v>-20</v>
+        <v>-10</v>
       </c>
       <c r="AI96" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="AJ96" t="n">
-        <v>0</v>
+        <v>-80</v>
       </c>
       <c r="AK96" t="n">
         <v>20</v>
@@ -15711,7 +15711,7 @@
       </c>
       <c r="AN96" t="inlineStr">
         <is>
-          <t>DT尚未轉強、尚未站上5MA、均線多頭排列、位於20日區間中上緣</t>
+          <t>DT尚未轉強、貼近5MA、位置偏低但需等轉強、分數轉弱</t>
         </is>
       </c>
       <c r="AO96" t="inlineStr">
@@ -15726,29 +15726,29 @@
       </c>
       <c r="AQ96" t="inlineStr">
         <is>
-          <t>跌破5日線、多頭排列、量能未放大</t>
+          <t>站上5日線、空頭排列、量能未放大、接近20日低點</t>
         </is>
       </c>
       <c r="AR96" t="inlineStr">
         <is>
-          <t>法人連續偏賣、5日法人明顯賣超、投信買外資賣</t>
+          <t>5日法人明顯賣超</t>
         </is>
       </c>
       <c r="AS96" t="inlineStr">
         <is>
-          <t>風險偏高：跌破5日線、多頭排列、量能未放大、法人連續偏賣、5日法人明顯賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
+          <t>風險偏高：站上5日線、空頭排列、量能未放大、接近20日低點、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>8028.TW</t>
+          <t>1303.TW</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>昇陽半導體</t>
+          <t>南亞</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -15757,28 +15757,28 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="E97" t="n">
-        <v>227.2</v>
+        <v>231.6</v>
       </c>
       <c r="F97" t="n">
-        <v>233.35</v>
+        <v>230.65</v>
       </c>
       <c r="G97" t="n">
-        <v>239.65</v>
+        <v>221.12</v>
       </c>
       <c r="H97" t="n">
-        <v>3815963</v>
+        <v>48008257</v>
       </c>
       <c r="I97" t="n">
-        <v>2975215</v>
+        <v>53361085</v>
       </c>
       <c r="J97" t="n">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="K97" t="n">
-        <v>216.5</v>
+        <v>174</v>
       </c>
       <c r="L97" t="inlineStr">
         <is>
@@ -15786,52 +15786,52 @@
         </is>
       </c>
       <c r="M97" t="n">
-        <v>-1407316</v>
+        <v>-3809309</v>
       </c>
       <c r="N97" t="n">
-        <v>-2439501</v>
+        <v>-22645671</v>
       </c>
       <c r="O97" t="n">
-        <v>-4015676</v>
+        <v>-26959115</v>
       </c>
       <c r="P97" t="n">
-        <v>-7292000</v>
+        <v>-37504582</v>
       </c>
       <c r="Q97" t="n">
-        <v>-1447130</v>
+        <v>-6798444</v>
       </c>
       <c r="R97" t="n">
-        <v>-3294271</v>
+        <v>-27265035</v>
       </c>
       <c r="S97" t="n">
-        <v>-4887144</v>
+        <v>-33056760</v>
       </c>
       <c r="T97" t="n">
-        <v>-8893544</v>
+        <v>-51665789</v>
       </c>
       <c r="U97" t="n">
-        <v>-2000</v>
+        <v>2714701</v>
       </c>
       <c r="V97" t="n">
-        <v>817000</v>
+        <v>5618279</v>
       </c>
       <c r="W97" t="n">
-        <v>852000</v>
+        <v>7877859</v>
       </c>
       <c r="X97" t="n">
-        <v>1696000</v>
+        <v>17968822</v>
       </c>
       <c r="Y97" t="n">
-        <v>41814</v>
+        <v>274434</v>
       </c>
       <c r="Z97" t="n">
-        <v>37770</v>
+        <v>-998915</v>
       </c>
       <c r="AA97" t="n">
-        <v>19468</v>
+        <v>-1780214</v>
       </c>
       <c r="AB97" t="n">
-        <v>-94456</v>
+        <v>-3807615</v>
       </c>
       <c r="AC97" t="n">
         <v>-20</v>
@@ -15849,28 +15849,28 @@
         <v>0</v>
       </c>
       <c r="AH97" t="n">
-        <v>-40</v>
+        <v>-20</v>
       </c>
       <c r="AI97" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ97" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK97" t="n">
         <v>20</v>
       </c>
-      <c r="AJ97" t="n">
-        <v>50</v>
-      </c>
-      <c r="AK97" t="n">
-        <v>55</v>
-      </c>
       <c r="AL97" t="n">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="AM97" t="inlineStr">
         <is>
-          <t>等待拉回確認</t>
+          <t>暫不追價</t>
         </is>
       </c>
       <c r="AN97" t="inlineStr">
         <is>
-          <t>DT尚未轉強、貼近5MA、量能溫和放大、分數明顯升溫</t>
+          <t>DT尚未轉強、尚未站上5MA、均線多頭排列、位於20日區間中上緣</t>
         </is>
       </c>
       <c r="AO97" t="inlineStr">
@@ -15885,7 +15885,7 @@
       </c>
       <c r="AQ97" t="inlineStr">
         <is>
-          <t>站上5日線、空頭排列、量能溫和放大</t>
+          <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
       <c r="AR97" t="inlineStr">
@@ -15895,7 +15895,7 @@
       </c>
       <c r="AS97" t="inlineStr">
         <is>
-          <t>風險偏高：站上5日線、空頭排列、量能溫和放大、法人連續偏賣、5日法人明顯賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
+          <t>風險偏高：跌破5日線、多頭排列、量能未放大、法人連續偏賣、5日法人明顯賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
@@ -19443,16 +19443,16 @@
         </is>
       </c>
       <c r="M120" t="n">
-        <v>-1782085</v>
+        <v>-1728375</v>
       </c>
       <c r="N120" t="n">
-        <v>-1363213</v>
+        <v>-1309503</v>
       </c>
       <c r="O120" t="n">
-        <v>-784287</v>
+        <v>-730577</v>
       </c>
       <c r="P120" t="n">
-        <v>5893017</v>
+        <v>5946727</v>
       </c>
       <c r="Q120" t="n">
         <v>-1483357</v>
@@ -19467,16 +19467,16 @@
         <v>6662166</v>
       </c>
       <c r="U120" t="n">
-        <v>-118000</v>
+        <v>-64290</v>
       </c>
       <c r="V120" t="n">
-        <v>-184000</v>
+        <v>-130290</v>
       </c>
       <c r="W120" t="n">
-        <v>-227000</v>
+        <v>-173290</v>
       </c>
       <c r="X120" t="n">
-        <v>-358200</v>
+        <v>-304490</v>
       </c>
       <c r="Y120" t="n">
         <v>-180728</v>
@@ -19602,16 +19602,16 @@
         </is>
       </c>
       <c r="M121" t="n">
-        <v>-627291</v>
+        <v>-636351</v>
       </c>
       <c r="N121" t="n">
-        <v>-1014141</v>
+        <v>-1023201</v>
       </c>
       <c r="O121" t="n">
-        <v>-1465152</v>
+        <v>-1474212</v>
       </c>
       <c r="P121" t="n">
-        <v>-3595388</v>
+        <v>-3604448</v>
       </c>
       <c r="Q121" t="n">
         <v>-349215</v>
@@ -19626,16 +19626,16 @@
         <v>-3650</v>
       </c>
       <c r="U121" t="n">
-        <v>-260000</v>
+        <v>-269060</v>
       </c>
       <c r="V121" t="n">
-        <v>-1133640</v>
+        <v>-1142700</v>
       </c>
       <c r="W121" t="n">
-        <v>-2350126</v>
+        <v>-2359186</v>
       </c>
       <c r="X121" t="n">
-        <v>-2890703</v>
+        <v>-2899763</v>
       </c>
       <c r="Y121" t="n">
         <v>-18076</v>
@@ -22303,16 +22303,16 @@
         </is>
       </c>
       <c r="M138" t="n">
-        <v>-6391165</v>
+        <v>-6070165</v>
       </c>
       <c r="N138" t="n">
-        <v>-2815955</v>
+        <v>-2494955</v>
       </c>
       <c r="O138" t="n">
-        <v>-10024427</v>
+        <v>-9703427</v>
       </c>
       <c r="P138" t="n">
-        <v>4532834</v>
+        <v>4853834</v>
       </c>
       <c r="Q138" t="n">
         <v>-6396915</v>
@@ -22327,16 +22327,16 @@
         <v>4870528</v>
       </c>
       <c r="U138" t="n">
-        <v>357020</v>
+        <v>678020</v>
       </c>
       <c r="V138" t="n">
-        <v>1294022</v>
+        <v>1615022</v>
       </c>
       <c r="W138" t="n">
-        <v>1643029</v>
+        <v>1964029</v>
       </c>
       <c r="X138" t="n">
-        <v>-67944</v>
+        <v>253056</v>
       </c>
       <c r="Y138" t="n">
         <v>-351270</v>

</xml_diff>